<commit_message>
push full project with push server
</commit_message>
<xml_diff>
--- a/stunden.xlsx
+++ b/stunden.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arikan\Documents\Software\echtebaerliner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656F14B9-B10D-443B-BC87-D0AB0F4DEBE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC07E7C-961F-4903-8556-04994FD207E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>x 25 €</t>
   </si>
@@ -45,13 +45,32 @@
   </si>
   <si>
     <t>0:30-2:30</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>13:00-14:30</t>
+  </si>
+  <si>
+    <t>15:00 - 16:30</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,15 +96,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Währung" xfId="1" builtinId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -363,13 +385,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>46080</v>
       </c>
@@ -380,14 +403,65 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="F1">
+      <c r="G1" s="2">
         <f>C1*25</f>
         <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46080</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>1.5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2">
+        <f>C2*25</f>
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>1.5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2">
+        <f>C3*25</f>
+        <v>37.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: include icon assets for expo build
</commit_message>
<xml_diff>
--- a/stunden.xlsx
+++ b/stunden.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arikan\Documents\Software\echtebaerliner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27103250-BA18-452A-9060-556E8B750C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC2D5B9-C808-4A3A-95BC-03EDDA2B7360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="7">
-  <si>
-    <t>x 25 €</t>
-  </si>
-  <si>
-    <t>=</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="13">
   <si>
     <t>0:30-2:30</t>
   </si>
@@ -56,7 +50,31 @@
     <t>15:00 - 16:30</t>
   </si>
   <si>
-    <t>14:00 - 15:00</t>
+    <t>18:30 - 20:30</t>
+  </si>
+  <si>
+    <t>Gesamt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:00 - 15:00 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:30 - 23:30 </t>
+  </si>
+  <si>
+    <t>aktueller stundensatz</t>
+  </si>
+  <si>
+    <t>11:00 - 13:00</t>
+  </si>
+  <si>
+    <t>15:30 - 16:30</t>
+  </si>
+  <si>
+    <t>17:45 - 18:15</t>
+  </si>
+  <si>
+    <t>14:00-15:00</t>
   </si>
 </sst>
 </file>
@@ -103,10 +121,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -388,108 +409,195 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>46080</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C1">
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="2">
-        <f>C1*25</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>46080</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C2">
         <v>1.5</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2">
-        <f>C2*25</f>
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2">
+        <f>1000/C14</f>
+        <v>57.142857142857146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>46082</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C3">
         <v>1.5</v>
       </c>
       <c r="D3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" t="s">
-        <v>0</v>
-      </c>
-      <c r="F3" t="s">
-        <v>1</v>
-      </c>
-      <c r="G3" s="2">
-        <f>C3*25</f>
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>46083</v>
       </c>
       <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C5">
         <v>3</v>
       </c>
-      <c r="E4" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="2">
-        <f>C4*25</f>
-        <v>25</v>
-      </c>
+      <c r="D5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>46090</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46091</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>46091</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9">
+        <v>0.5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14">
+        <f>SUM(C1:C13)</f>
+        <v>17.5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G19" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>